<commit_message>
Publish five certified Alder Ridge sample tasks
</commit_message>
<xml_diff>
--- a/environment/seed/sources/Shared/Finance/Close/2026/06 June/1 close mgmt/June close tracker - working - upd 7.1 810am.xlsx
+++ b/environment/seed/sources/Shared/Finance/Close/2026/06 June/1 close mgmt/June close tracker - working - upd 7.1 810am.xlsx
@@ -6,7 +6,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Close Calendar" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dependencies" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="late list + slack copy" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="chat copy 6.30-7.1" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="owner lookup OLD" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="June template - old" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
@@ -2393,7 +2393,7 @@
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>ARM-2409, ARM-2417 and ARM-2506</t>
+          <t>See current submission register for review queue</t>
         </is>
       </c>
     </row>
@@ -2553,7 +2553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -2567,7 +2567,7 @@
     <row r="1">
       <c r="A1" s="9" t="inlineStr">
         <is>
-          <t>Manually copied from close chat 6/30-7/1. Duplicate lines were not removed because replies sometimes contain the actual resolution.</t>
+          <t>Manually copied from close chat 6/30-7/1. Duplicate lines were retained where the reply context was unclear.</t>
         </is>
       </c>
     </row>
@@ -2654,7 +2654,7 @@
       </c>
       <c r="D5" s="11" t="inlineStr">
         <is>
-          <t>Does that include the Northline concrete rework?</t>
+          <t>Warehouse issue batch was submitted after the afternoon report pull</t>
         </is>
       </c>
       <c r="E5" s="11" t="inlineStr">
@@ -2682,7 +2682,7 @@
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>No - that's in the subcontractor dispute file, cost is already posted</t>
+          <t>Receiving team is checking the remaining unmatched slips</t>
         </is>
       </c>
       <c r="E6" s="11" t="inlineStr">
@@ -2692,7 +2692,7 @@
       </c>
       <c r="F6" s="11" t="inlineStr">
         <is>
-          <t>y</t>
+          <t>n</t>
         </is>
       </c>
     </row>
@@ -2731,7 +2731,7 @@
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>7/1 7:41a</t>
+          <t>7/1 7:28a</t>
         </is>
       </c>
       <c r="B8" s="11" t="inlineStr">
@@ -2746,7 +2746,7 @@
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>Need PM follow-up on 2409/2417/2506 before noon</t>
+          <t>Columbia — MC/NB huddle done after yesterday's site note. Keep the lift/retest cost basis; 029 stays out.</t>
         </is>
       </c>
       <c r="E8" s="11" t="inlineStr">
@@ -2756,69 +2756,101 @@
       </c>
       <c r="F8" s="11" t="inlineStr">
         <is>
-          <t>n</t>
+          <t>y</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="11" t="inlineStr">
         <is>
+          <t>7/1 7:41a</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>WIP</t>
+        </is>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>Need owners on low-confidence PM submissions before noon</t>
+        </is>
+      </c>
+      <c r="E9" s="11" t="inlineStr">
+        <is>
+          <t>KS</t>
+        </is>
+      </c>
+      <c r="F9" s="11" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
           <t>7/1 8:06a</t>
         </is>
       </c>
-      <c r="B9" s="11" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>DC</t>
         </is>
       </c>
-      <c r="C9" s="11" t="inlineStr">
+      <c r="C10" s="11" t="inlineStr">
         <is>
           <t>reporting</t>
         </is>
       </c>
-      <c r="D9" s="11" t="inlineStr">
+      <c r="D10" s="11" t="inlineStr">
         <is>
           <t>May deck marked final is okay for style, not for June numbers</t>
         </is>
       </c>
-      <c r="E9" s="11" t="inlineStr">
+      <c r="E10" s="11" t="inlineStr">
         <is>
           <t>MB</t>
         </is>
       </c>
-      <c r="F9" s="11" t="inlineStr">
+      <c r="F10" s="11" t="inlineStr">
         <is>
           <t>FYI</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="12" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
         <is>
           <t>7/1 8:09a</t>
         </is>
       </c>
-      <c r="B10" s="12" t="inlineStr">
+      <c r="B11" s="12" t="inlineStr">
         <is>
           <t>NB</t>
         </is>
       </c>
-      <c r="C10" s="12" t="inlineStr">
+      <c r="C11" s="12" t="inlineStr">
         <is>
           <t>close</t>
         </is>
       </c>
-      <c r="D10" s="12" t="inlineStr">
+      <c r="D11" s="12" t="inlineStr">
         <is>
           <t>readme updated in folder</t>
         </is>
       </c>
-      <c r="E10" s="12" t="inlineStr">
+      <c r="E11" s="12" t="inlineStr">
         <is>
           <t>NB</t>
         </is>
       </c>
-      <c r="F10" s="12" t="inlineStr">
+      <c r="F11" s="12" t="inlineStr">
         <is>
           <t>y</t>
         </is>
@@ -2976,7 +3008,7 @@
       </c>
       <c r="F6" s="11" t="inlineStr">
         <is>
-          <t>late receiving can move job cost</t>
+          <t>review the current intake and receiving queues</t>
         </is>
       </c>
     </row>

</xml_diff>